<commit_message>
Cierre de vacíos de la v6, gráfico integrado y modelos de certificación
Resuelve en el Anexo 2 los vacíos de la revisión v6 (PD-02, VI-05,
desglose de Avanciencia, vinculaciones, poder e interés, firmantes del
plan de sostenibilidad, ventana de compra del laboratorio y respaldo del
bucle de adopción), agrega el gráfico integrado del proyecto y los
modelos de certificación de contrapartida.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DeWH6PkcBrmc83oq5HNaqd
</commit_message>
<xml_diff>
--- a/genesis-e4-e3p00/ANEXO_2/v6_alianza_cinco/matriz_correspondencia_v6.xlsx
+++ b/genesis-e4-e3p00/ANEXO_2/v6_alianza_cinco/matriz_correspondencia_v6.xlsx
@@ -8655,7 +8655,7 @@
       </c>
       <c r="U83" s="4" t="inlineStr">
         <is>
-          <t>El Anexo 3 declara cotizaciones pendientes (TdR 12.2: al menos dos por rubro, no subsanable) | El Anexo 3 v6 programa la partida en la actividad 1.1 (meses 2 a 4); el Plan de transferencia ejecuta horas de asesoría hasta el mes 23: confirmar el perfil de pagos</t>
+          <t>El Anexo 3 declara cotizaciones pendientes (TdR 12.2: al menos dos por rubro, no subsanable) | Las 150 horas se ejecutan en M2–M4 (actividad 1.1); la aplicación posterior la ejecutan TH-16 y TH-22 de Avanciencia sin costo adicional de esta línea (tabla 18.5)</t>
         </is>
       </c>
     </row>
@@ -9920,7 +9920,7 @@
       </c>
       <c r="U96" s="4" t="inlineStr">
         <is>
-          <t>El Anexo 3 v6 asigna la partida a la actividad 2.3; su concepto cubre los tramos 2 y 3 (actividades 2.3 y 2.4)</t>
+          <t>Partida completa en su actividad principal (2.3), según la regla del cronograma financiero; también financia la instalación del tramo 3 (2.4)</t>
         </is>
       </c>
     </row>
@@ -11539,12 +11539,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>La consulta de libertad de operación precede a la compra del lote 1, pero el Plan de transferencia programa asesoría hasta el mes 23</t>
+          <t>Resuelto: las 150 horas producen en M2–M4 el informe de libertad de operación, el borrador del acuerdo marco, las minutas de convenio y la matriz de vencimientos; la aplicación posterior la ejecutan TH-16 y TH-22 de Avanciencia (tabla 18.5)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Confirmar si el contrato se paga en M2–M4 con entregas posteriores o extender el perfil de pagos</t>
+          <t>Sin ajuste al Anexo 3</t>
         </is>
       </c>
     </row>

</xml_diff>